<commit_message>
Rebuild candidate list from new SOS file, fix 10 race/district mismatches, merge duplicates
</commit_message>
<xml_diff>
--- a/viz/data/clean/US_House_D1_ALL_Transactions.xlsx
+++ b/viz/data/clean/US_House_D1_ALL_Transactions.xlsx
@@ -7,8 +7,8 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Receipts" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Expenditures" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Receipts" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="All Expenditures" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -40689,7 +40689,7 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
-          <t>Purpose Category</t>
+          <t>Purpose</t>
         </is>
       </c>
     </row>

</xml_diff>